<commit_message>
Added MCA in the workflow,now we can upload pdf from UI and generate summary for Companies act every week
</commit_message>
<xml_diff>
--- a/data/Links_test.xlsx
+++ b/data/Links_test.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
   <si>
     <t>IBBI - Litigation</t>
   </si>
@@ -29,16 +29,10 @@
     <t>IFSCA</t>
   </si>
   <si>
-    <t>Public Consultation</t>
-  </si>
-  <si>
-    <t>https://ifsca.gov.in/ReportPublication/index/sKCVtbX6J9o=</t>
+    <t/>
   </si>
   <si>
     <t>Listed Companies</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>SEBI</t>
@@ -162,6 +156,12 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -169,12 +169,6 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
@@ -522,7 +516,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -551,7 +545,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1"/>
-      <c r="B2" s="9"/>
+      <c r="B2" s="11"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -691,7 +685,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1"/>
-      <c r="B7" s="9"/>
+      <c r="B7" s="11"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -28535,7 +28529,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="10" width="61.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="61.43357142857143" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="5" width="13.005" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="5" width="13.005" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="5" width="13.005" customWidth="1" bestFit="1"/>
@@ -28560,7 +28554,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -28583,12 +28577,8 @@
       <c r="U1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>6</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -28610,12 +28600,8 @@
       <c r="U2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
-      <c r="A3" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>6</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -51604,7 +51590,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="10" width="40.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="40.57642857142857" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -51613,12 +51599,12 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
+      <c r="A2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>4</v>
+      <c r="B2" s="9" t="s">
+        <v>3</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
@@ -51634,20 +51620,20 @@
       <c r="B5" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="8"/>
+      <c r="A6" s="10"/>
       <c r="B6" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="8"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="8"/>
+      <c r="A8" s="10"/>
       <c r="B8" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1"/>
-      <c r="B9" s="9"/>
+      <c r="B9" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added acts into parsing agents
</commit_message>
<xml_diff>
--- a/data/Links_test.xlsx
+++ b/data/Links_test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Companies Act"/>
@@ -23,6 +23,9 @@
     <t>IBBI - Litigation</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>RBI</t>
   </si>
   <si>
@@ -34,9 +37,6 @@
   <si>
     <t xml:space="preserve">Companies Act
 </t>
-  </si>
-  <si>
-    <t/>
   </si>
 </sst>
 </file>
@@ -81,12 +81,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFd9ead3"/>
+        <fgColor rgb="FFf4cccc"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFf4cccc"/>
+        <fgColor rgb="FFd9ead3"/>
       </patternFill>
     </fill>
     <fill>
@@ -142,16 +142,22 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
@@ -174,12 +180,6 @@
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -486,38 +486,38 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="75.14785714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="75.14785714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="7" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -544,13 +544,9 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>5</v>
-      </c>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="1"/>
+      <c r="B2" s="5"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -578,7 +574,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1"/>
-      <c r="B3" s="3"/>
+      <c r="B3" s="5"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -606,7 +602,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1"/>
-      <c r="B4" s="3"/>
+      <c r="B4" s="5"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -634,7 +630,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1"/>
-      <c r="B5" s="3"/>
+      <c r="B5" s="5"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -662,7 +658,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1"/>
-      <c r="B6" s="3"/>
+      <c r="B6" s="5"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -690,7 +686,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1"/>
-      <c r="B7" s="9"/>
+      <c r="B7" s="11"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -28533,33 +28529,33 @@
   <dimension ref="A1:U1001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="10" width="61.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="61.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="7" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -28583,7 +28579,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1"/>
-      <c r="B2" s="3"/>
+      <c r="B2" s="5"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -28606,7 +28602,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
       <c r="A3" s="1"/>
-      <c r="B3" s="3"/>
+      <c r="B3" s="5"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -28628,8 +28624,8 @@
       <c r="U3" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="11"/>
-      <c r="B4" s="12"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="14"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -51533,53 +51529,53 @@
       <c r="R999" s="1"/>
       <c r="S999" s="1"/>
       <c r="T999" s="1"/>
-      <c r="U999" s="11"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="18" customFormat="1" s="13">
-      <c r="A1000" s="12"/>
+      <c r="U999" s="13"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="18" customFormat="1" s="15">
+      <c r="A1000" s="14"/>
       <c r="B1000" s="2"/>
-      <c r="C1000" s="12"/>
-      <c r="D1000" s="12"/>
-      <c r="E1000" s="12"/>
-      <c r="F1000" s="12"/>
-      <c r="G1000" s="12"/>
-      <c r="H1000" s="12"/>
-      <c r="I1000" s="12"/>
-      <c r="J1000" s="12"/>
-      <c r="K1000" s="12"/>
-      <c r="L1000" s="12"/>
-      <c r="M1000" s="12"/>
-      <c r="N1000" s="12"/>
-      <c r="O1000" s="12"/>
-      <c r="P1000" s="12"/>
-      <c r="Q1000" s="12"/>
-      <c r="R1000" s="12"/>
-      <c r="S1000" s="12"/>
-      <c r="T1000" s="12"/>
-      <c r="U1000" s="12"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="18" customFormat="1" s="13">
-      <c r="A1001" s="12"/>
+      <c r="C1000" s="14"/>
+      <c r="D1000" s="14"/>
+      <c r="E1000" s="14"/>
+      <c r="F1000" s="14"/>
+      <c r="G1000" s="14"/>
+      <c r="H1000" s="14"/>
+      <c r="I1000" s="14"/>
+      <c r="J1000" s="14"/>
+      <c r="K1000" s="14"/>
+      <c r="L1000" s="14"/>
+      <c r="M1000" s="14"/>
+      <c r="N1000" s="14"/>
+      <c r="O1000" s="14"/>
+      <c r="P1000" s="14"/>
+      <c r="Q1000" s="14"/>
+      <c r="R1000" s="14"/>
+      <c r="S1000" s="14"/>
+      <c r="T1000" s="14"/>
+      <c r="U1000" s="14"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="18" customFormat="1" s="15">
+      <c r="A1001" s="14"/>
       <c r="B1001" s="2"/>
-      <c r="C1001" s="12"/>
-      <c r="D1001" s="12"/>
-      <c r="E1001" s="12"/>
-      <c r="F1001" s="12"/>
-      <c r="G1001" s="12"/>
-      <c r="H1001" s="12"/>
-      <c r="I1001" s="12"/>
-      <c r="J1001" s="12"/>
-      <c r="K1001" s="12"/>
-      <c r="L1001" s="12"/>
-      <c r="M1001" s="12"/>
-      <c r="N1001" s="12"/>
-      <c r="O1001" s="12"/>
-      <c r="P1001" s="12"/>
-      <c r="Q1001" s="12"/>
-      <c r="R1001" s="12"/>
-      <c r="S1001" s="12"/>
-      <c r="T1001" s="12"/>
-      <c r="U1001" s="12"/>
+      <c r="C1001" s="14"/>
+      <c r="D1001" s="14"/>
+      <c r="E1001" s="14"/>
+      <c r="F1001" s="14"/>
+      <c r="G1001" s="14"/>
+      <c r="H1001" s="14"/>
+      <c r="I1001" s="14"/>
+      <c r="J1001" s="14"/>
+      <c r="K1001" s="14"/>
+      <c r="L1001" s="14"/>
+      <c r="M1001" s="14"/>
+      <c r="N1001" s="14"/>
+      <c r="O1001" s="14"/>
+      <c r="P1001" s="14"/>
+      <c r="Q1001" s="14"/>
+      <c r="R1001" s="14"/>
+      <c r="S1001" s="14"/>
+      <c r="T1001" s="14"/>
+      <c r="U1001" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51594,47 +51590,47 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="10" width="40.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="40.57642857142857" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1"/>
-      <c r="B2" s="3"/>
+      <c r="B2" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1"/>
-      <c r="B3" s="3"/>
+      <c r="B3" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1"/>
-      <c r="B4" s="3"/>
+      <c r="B4" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1"/>
-      <c r="B5" s="3"/>
+      <c r="B5" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="8"/>
-      <c r="B6" s="3"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="8"/>
-      <c r="B7" s="3"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="8"/>
-      <c r="B8" s="3"/>
+      <c r="A8" s="10"/>
+      <c r="B8" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1"/>
-      <c r="B9" s="9"/>
+      <c r="B9" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51649,39 +51645,39 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="48.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="48.86214285714286" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="6"/>
-      <c r="B2" s="3"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="7"/>
-      <c r="B3" s="3"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="6"/>
-      <c r="B4" s="3"/>
+      <c r="A4" s="8"/>
+      <c r="B4" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="7"/>
-      <c r="B5" s="3"/>
+      <c r="A5" s="9"/>
+      <c r="B5" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="6"/>
-      <c r="B6" s="3"/>
+      <c r="A6" s="8"/>
+      <c r="B6" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="6"/>
-      <c r="B7" s="3"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1"/>
@@ -51700,8 +51696,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="41.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="41.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
@@ -51711,28 +51707,32 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="1"/>
-      <c r="B2" s="3"/>
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
       <c r="A3" s="1"/>
-      <c r="B3" s="3"/>
+      <c r="B3" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
       <c r="A4" s="1"/>
-      <c r="B4" s="3"/>
+      <c r="B4" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
       <c r="A5" s="1"/>
-      <c r="B5" s="4"/>
+      <c r="B5" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
       <c r="A6" s="1"/>
-      <c r="B6" s="4"/>
+      <c r="B6" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
       <c r="A7" s="1"/>
-      <c r="B7" s="3"/>
+      <c r="B7" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added ifsca acts to links
</commit_message>
<xml_diff>
--- a/data/Links_test.xlsx
+++ b/data/Links_test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="4"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Companies Act"/>
@@ -23,13 +23,13 @@
     <t>IBBI - Litigation</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>RBI</t>
   </si>
   <si>
     <t>IFSCA</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>Listed Companies</t>
@@ -142,11 +142,8 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -157,11 +154,14 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -486,32 +486,32 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="75.14785714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="75.14785714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="6" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -546,7 +546,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1"/>
-      <c r="B2" s="5"/>
+      <c r="B2" s="4"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -574,7 +574,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1"/>
-      <c r="B3" s="5"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -602,7 +602,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1"/>
-      <c r="B4" s="5"/>
+      <c r="B4" s="4"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -630,7 +630,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1"/>
-      <c r="B5" s="5"/>
+      <c r="B5" s="4"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -658,7 +658,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1"/>
-      <c r="B6" s="5"/>
+      <c r="B6" s="4"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -936,7 +936,7 @@
       <c r="Y15" s="1"/>
       <c r="Z15" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -964,7 +964,7 @@
       <c r="Y16" s="1"/>
       <c r="Z16" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -992,7 +992,7 @@
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1020,7 +1020,7 @@
       <c r="Y18" s="1"/>
       <c r="Z18" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1048,7 +1048,7 @@
       <c r="Y19" s="1"/>
       <c r="Z19" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -28529,27 +28529,27 @@
   <dimension ref="A1:U1001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="13.005" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="12" width="61.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="6" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -28579,7 +28579,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1"/>
-      <c r="B2" s="5"/>
+      <c r="B2" s="4"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -28602,7 +28602,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
       <c r="A3" s="1"/>
-      <c r="B3" s="5"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -51590,43 +51590,47 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="13.005" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="12" width="40.57642857142857" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
+      <c r="A2" s="8" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1"/>
-      <c r="B2" s="5"/>
+      <c r="B2" s="9" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1"/>
-      <c r="B3" s="5"/>
+      <c r="B3" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1"/>
-      <c r="B4" s="5"/>
+      <c r="B4" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1"/>
-      <c r="B5" s="5"/>
+      <c r="B5" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="10"/>
-      <c r="B6" s="5"/>
+      <c r="B6" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="10"/>
-      <c r="B7" s="5"/>
+      <c r="B7" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="10"/>
-      <c r="B8" s="5"/>
+      <c r="B8" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1"/>
@@ -51645,39 +51649,39 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="48.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="48.86214285714286" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="8"/>
-      <c r="B2" s="5"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="9"/>
-      <c r="B3" s="5"/>
+      <c r="A3" s="7"/>
+      <c r="B3" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="8"/>
-      <c r="B4" s="5"/>
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="9"/>
-      <c r="B5" s="5"/>
+      <c r="A5" s="7"/>
+      <c r="B5" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="8"/>
-      <c r="B6" s="5"/>
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="8"/>
-      <c r="B7" s="5"/>
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1"/>
@@ -51696,8 +51700,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="41.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="41.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
@@ -51707,32 +51711,28 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
       <c r="A3" s="1"/>
-      <c r="B3" s="5"/>
+      <c r="B3" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
       <c r="A4" s="1"/>
-      <c r="B4" s="5"/>
+      <c r="B4" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
       <c r="A5" s="1"/>
-      <c r="B5" s="6"/>
+      <c r="B5" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
       <c r="A6" s="1"/>
-      <c r="B6" s="6"/>
+      <c r="B6" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
       <c r="A7" s="1"/>
-      <c r="B7" s="5"/>
+      <c r="B7" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated,rbi has blocked windows system
</commit_message>
<xml_diff>
--- a/data/Links_test.xlsx
+++ b/data/Links_test.xlsx
@@ -18,12 +18,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t>IBBI - Litigation</t>
   </si>
   <si>
     <t>RBI</t>
+  </si>
+  <si>
+    <t>Notifications</t>
+  </si>
+  <si>
+    <t>https://www.rbi.org.in/Scripts/NotificationUser.aspx</t>
+  </si>
+  <si>
+    <t>Press Release</t>
+  </si>
+  <si>
+    <t>https://www.rbi.org.in/Scripts/BS_PressReleaseDisplay.aspx</t>
   </si>
   <si>
     <t>IFSCA</t>
@@ -32,17 +44,11 @@
     <t>Listed Companies</t>
   </si>
   <si>
-    <t>Circular-BSE</t>
-  </si>
-  <si>
-    <t>https://www.bseindia.com/corporates/CirularToListedComp.html</t>
+    <t/>
   </si>
   <si>
     <t xml:space="preserve">Companies Act
 </t>
-  </si>
-  <si>
-    <t/>
   </si>
 </sst>
 </file>
@@ -172,6 +178,12 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -180,12 +192,6 @@
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -523,7 +529,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -551,12 +557,8 @@
       <c r="Z1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>7</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="4"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -28565,7 +28567,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -28588,11 +28590,11 @@
       <c r="U1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
+      <c r="A2" s="11" t="s">
+        <v>8</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>5</v>
+      <c r="B2" s="12" t="s">
+        <v>8</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -28638,8 +28640,8 @@
       <c r="U3" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="11"/>
-      <c r="B4" s="12"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="14"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -51543,53 +51545,53 @@
       <c r="R999" s="1"/>
       <c r="S999" s="1"/>
       <c r="T999" s="1"/>
-      <c r="U999" s="11"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="18" customFormat="1" s="13">
-      <c r="A1000" s="12"/>
+      <c r="U999" s="13"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="18" customFormat="1" s="15">
+      <c r="A1000" s="14"/>
       <c r="B1000" s="2"/>
-      <c r="C1000" s="12"/>
-      <c r="D1000" s="12"/>
-      <c r="E1000" s="12"/>
-      <c r="F1000" s="12"/>
-      <c r="G1000" s="12"/>
-      <c r="H1000" s="12"/>
-      <c r="I1000" s="12"/>
-      <c r="J1000" s="12"/>
-      <c r="K1000" s="12"/>
-      <c r="L1000" s="12"/>
-      <c r="M1000" s="12"/>
-      <c r="N1000" s="12"/>
-      <c r="O1000" s="12"/>
-      <c r="P1000" s="12"/>
-      <c r="Q1000" s="12"/>
-      <c r="R1000" s="12"/>
-      <c r="S1000" s="12"/>
-      <c r="T1000" s="12"/>
-      <c r="U1000" s="12"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="18" customFormat="1" s="13">
-      <c r="A1001" s="12"/>
+      <c r="C1000" s="14"/>
+      <c r="D1000" s="14"/>
+      <c r="E1000" s="14"/>
+      <c r="F1000" s="14"/>
+      <c r="G1000" s="14"/>
+      <c r="H1000" s="14"/>
+      <c r="I1000" s="14"/>
+      <c r="J1000" s="14"/>
+      <c r="K1000" s="14"/>
+      <c r="L1000" s="14"/>
+      <c r="M1000" s="14"/>
+      <c r="N1000" s="14"/>
+      <c r="O1000" s="14"/>
+      <c r="P1000" s="14"/>
+      <c r="Q1000" s="14"/>
+      <c r="R1000" s="14"/>
+      <c r="S1000" s="14"/>
+      <c r="T1000" s="14"/>
+      <c r="U1000" s="14"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="18" customFormat="1" s="15">
+      <c r="A1001" s="14"/>
       <c r="B1001" s="2"/>
-      <c r="C1001" s="12"/>
-      <c r="D1001" s="12"/>
-      <c r="E1001" s="12"/>
-      <c r="F1001" s="12"/>
-      <c r="G1001" s="12"/>
-      <c r="H1001" s="12"/>
-      <c r="I1001" s="12"/>
-      <c r="J1001" s="12"/>
-      <c r="K1001" s="12"/>
-      <c r="L1001" s="12"/>
-      <c r="M1001" s="12"/>
-      <c r="N1001" s="12"/>
-      <c r="O1001" s="12"/>
-      <c r="P1001" s="12"/>
-      <c r="Q1001" s="12"/>
-      <c r="R1001" s="12"/>
-      <c r="S1001" s="12"/>
-      <c r="T1001" s="12"/>
-      <c r="U1001" s="12"/>
+      <c r="C1001" s="14"/>
+      <c r="D1001" s="14"/>
+      <c r="E1001" s="14"/>
+      <c r="F1001" s="14"/>
+      <c r="G1001" s="14"/>
+      <c r="H1001" s="14"/>
+      <c r="I1001" s="14"/>
+      <c r="J1001" s="14"/>
+      <c r="K1001" s="14"/>
+      <c r="L1001" s="14"/>
+      <c r="M1001" s="14"/>
+      <c r="N1001" s="14"/>
+      <c r="O1001" s="14"/>
+      <c r="P1001" s="14"/>
+      <c r="Q1001" s="14"/>
+      <c r="R1001" s="14"/>
+      <c r="S1001" s="14"/>
+      <c r="T1001" s="14"/>
+      <c r="U1001" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51611,7 +51613,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
@@ -51670,12 +51672,20 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="3"/>
-      <c r="B2" s="4"/>
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="7"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="3"/>

</xml_diff>

<commit_message>
fixed informal guidance title issue of sebi
</commit_message>
<xml_diff>
--- a/data/Links_test.xlsx
+++ b/data/Links_test.xlsx
@@ -4,13 +4,13 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="RBI"/>
+    <sheet r:id="rId1" sheetId="1" name="SEBI"/>
     <sheet r:id="rId2" sheetId="2" name="Listed Companies"/>
     <sheet r:id="rId3" sheetId="3" name="Companies Act"/>
-    <sheet r:id="rId4" sheetId="4" name="ICAI"/>
+    <sheet r:id="rId4" sheetId="4" name="RBI"/>
     <sheet r:id="rId5" sheetId="5" name="IFSCA"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
@@ -30,13 +30,13 @@
 </t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Listed Companies</t>
   </si>
   <si>
     <t>RBI</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -163,12 +163,6 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -177,6 +171,12 @@
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -493,22 +493,26 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="13" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="3"/>
-      <c r="B2" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
+      <c r="B2" s="14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="15"/>
       <c r="B3" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="31.5">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="15"/>
       <c r="B5" s="4"/>
     </row>
@@ -563,7 +567,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -632,8 +636,8 @@
       <c r="U3" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="12"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="11"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -23537,53 +23541,53 @@
       <c r="R999" s="1"/>
       <c r="S999" s="1"/>
       <c r="T999" s="1"/>
-      <c r="U999" s="12"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="18" customFormat="1" s="14">
-      <c r="A1000" s="13"/>
+      <c r="U999" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1000" customHeight="1" ht="18" customFormat="1" s="12">
+      <c r="A1000" s="11"/>
       <c r="B1000" s="2"/>
-      <c r="C1000" s="13"/>
-      <c r="D1000" s="13"/>
-      <c r="E1000" s="13"/>
-      <c r="F1000" s="13"/>
-      <c r="G1000" s="13"/>
-      <c r="H1000" s="13"/>
-      <c r="I1000" s="13"/>
-      <c r="J1000" s="13"/>
-      <c r="K1000" s="13"/>
-      <c r="L1000" s="13"/>
-      <c r="M1000" s="13"/>
-      <c r="N1000" s="13"/>
-      <c r="O1000" s="13"/>
-      <c r="P1000" s="13"/>
-      <c r="Q1000" s="13"/>
-      <c r="R1000" s="13"/>
-      <c r="S1000" s="13"/>
-      <c r="T1000" s="13"/>
-      <c r="U1000" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="18" customFormat="1" s="14">
-      <c r="A1001" s="13"/>
+      <c r="C1000" s="11"/>
+      <c r="D1000" s="11"/>
+      <c r="E1000" s="11"/>
+      <c r="F1000" s="11"/>
+      <c r="G1000" s="11"/>
+      <c r="H1000" s="11"/>
+      <c r="I1000" s="11"/>
+      <c r="J1000" s="11"/>
+      <c r="K1000" s="11"/>
+      <c r="L1000" s="11"/>
+      <c r="M1000" s="11"/>
+      <c r="N1000" s="11"/>
+      <c r="O1000" s="11"/>
+      <c r="P1000" s="11"/>
+      <c r="Q1000" s="11"/>
+      <c r="R1000" s="11"/>
+      <c r="S1000" s="11"/>
+      <c r="T1000" s="11"/>
+      <c r="U1000" s="11"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="18" customFormat="1" s="12">
+      <c r="A1001" s="11"/>
       <c r="B1001" s="2"/>
-      <c r="C1001" s="13"/>
-      <c r="D1001" s="13"/>
-      <c r="E1001" s="13"/>
-      <c r="F1001" s="13"/>
-      <c r="G1001" s="13"/>
-      <c r="H1001" s="13"/>
-      <c r="I1001" s="13"/>
-      <c r="J1001" s="13"/>
-      <c r="K1001" s="13"/>
-      <c r="L1001" s="13"/>
-      <c r="M1001" s="13"/>
-      <c r="N1001" s="13"/>
-      <c r="O1001" s="13"/>
-      <c r="P1001" s="13"/>
-      <c r="Q1001" s="13"/>
-      <c r="R1001" s="13"/>
-      <c r="S1001" s="13"/>
-      <c r="T1001" s="13"/>
-      <c r="U1001" s="13"/>
+      <c r="C1001" s="11"/>
+      <c r="D1001" s="11"/>
+      <c r="E1001" s="11"/>
+      <c r="F1001" s="11"/>
+      <c r="G1001" s="11"/>
+      <c r="H1001" s="11"/>
+      <c r="I1001" s="11"/>
+      <c r="J1001" s="11"/>
+      <c r="K1001" s="11"/>
+      <c r="L1001" s="11"/>
+      <c r="M1001" s="11"/>
+      <c r="N1001" s="11"/>
+      <c r="O1001" s="11"/>
+      <c r="P1001" s="11"/>
+      <c r="Q1001" s="11"/>
+      <c r="R1001" s="11"/>
+      <c r="S1001" s="11"/>
+      <c r="T1001" s="11"/>
+      <c r="U1001" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23657,12 +23661,8 @@
       <c r="Z1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
-      <c r="A2" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>3</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="4"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>

</xml_diff>